<commit_message>
Added attendance predictor, bunk planner, productivity score and email reminder system
</commit_message>
<xml_diff>
--- a/data/database.xlsx
+++ b/data/database.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" tabRatio="600" firstSheet="1" activeTab="6" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Attendance" sheetId="1" state="visible" r:id="rId1"/>
@@ -15,7 +16,7 @@
     <sheet name="Tasks" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -24,18 +25,13 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
@@ -49,27 +45,12 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -82,19 +63,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -457,8 +435,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -508,6 +486,57 @@
       <c r="C3" t="inlineStr">
         <is>
           <t>Period 5 (18:55 – 20:00)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Period 1 (10:00 – 10:55)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Period 2 (10:55 – 11:50)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Period 3 (12:05 – 13:00)</t>
         </is>
       </c>
     </row>
@@ -522,26 +551,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>subject</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>minutes</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>date</t>
         </is>
@@ -561,7 +590,7 @@
       <c r="C2" t="n">
         <v>15</v>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D2" s="3" t="n">
         <v>46061</v>
       </c>
     </row>
@@ -579,7 +608,7 @@
       <c r="C3" t="n">
         <v>30</v>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" s="3" t="n">
         <v>46061</v>
       </c>
     </row>
@@ -597,7 +626,7 @@
       <c r="C4" t="n">
         <v>50</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="3" t="n">
         <v>46068</v>
       </c>
     </row>
@@ -615,7 +644,7 @@
       <c r="C5" t="n">
         <v>16</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="3" t="n">
         <v>46069</v>
       </c>
     </row>
@@ -633,8 +662,26 @@
       <c r="C6" t="n">
         <v>21</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="3" t="n">
         <v>46069</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>dcn</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>11</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>46082</v>
       </c>
     </row>
   </sheetData>
@@ -652,17 +699,17 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>habit</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>date</t>
         </is>
@@ -853,7 +900,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>habit</t>
         </is>
@@ -899,7 +946,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -964,27 +1011,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>attendance</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>monthlygoal</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>minattendance</t>
         </is>
@@ -1022,36 +1069,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Created_Date</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Last_Reminded</t>
         </is>
@@ -1065,12 +1112,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>nxt</t>
+          <t>a</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1080,12 +1127,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-02-16 07:41:21</t>
+          <t>2026-03-01 16:30:51</t>
         </is>
       </c>
     </row>
@@ -1097,7 +1144,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>f</t>
+          <t>aa</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1112,12 +1159,44 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-02-16 07:57:01</t>
+          <t>2026-03-01 19:37:25</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ad</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-03-01 12:48:55</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Updated attendance period timing (1PM to 6PM schedule)
</commit_message>
<xml_diff>
--- a/data/database.xlsx
+++ b/data/database.xlsx
@@ -1069,7 +1069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1200,6 +1200,38 @@
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>re9</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>2026-03-01</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-03-01 21:02:23</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
i think it is the last update thankyou !!!
</commit_message>
<xml_diff>
--- a/data/database.xlsx
+++ b/data/database.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-23148" yWindow="-1308" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Attendance" sheetId="1" state="visible" r:id="rId1"/>
@@ -16,22 +15,34 @@
     <sheet name="Tasks" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
+  <numFmts count="3">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
     <font>
       <b val="1"/>
@@ -45,12 +56,42 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -63,16 +104,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -435,8 +483,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:C14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
+  <cols>
+    <col width="13.33203125" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
@@ -461,14 +512,12 @@
           <t>manishmanoj006@gmail.com</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-02-08</t>
-        </is>
+      <c r="B2" s="2" t="n">
+        <v>46086</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Period 4 (18:00 – 18:55)</t>
+          <t xml:space="preserve">Period 4 </t>
         </is>
       </c>
     </row>
@@ -478,14 +527,12 @@
           <t>manishmanoj006@gmail.com</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-02-08</t>
-        </is>
+      <c r="B3" s="2" t="n">
+        <v>46086</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Period 5 (18:55 – 20:00)</t>
+          <t xml:space="preserve">Period 5 </t>
         </is>
       </c>
     </row>
@@ -495,14 +542,12 @@
           <t>manishmanoj006@gmail.com</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
+      <c r="B4" s="2" t="n">
+        <v>46087</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Period 1 (10:00 – 10:55)</t>
+          <t xml:space="preserve">Period 1 </t>
         </is>
       </c>
     </row>
@@ -512,14 +557,12 @@
           <t>manishmanoj006@gmail.com</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
+      <c r="B5" s="2" t="n">
+        <v>46087</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Period 2 (10:55 – 11:50)</t>
+          <t xml:space="preserve">Period 2 </t>
         </is>
       </c>
     </row>
@@ -529,14 +572,132 @@
           <t>manishmanoj006@gmail.com</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
+      <c r="B6" s="2" t="n">
+        <v>46087</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Period 3 (12:05 – 13:00)</t>
+          <t xml:space="preserve">Period 3 </t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>46088</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Period 1 </t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>46088</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Period 2 </t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>46088</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Period 3 </t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>46089</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Period 1 </t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>46089</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Period 2 </t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>46089</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Period 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>46089</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Period 4 </t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>46089</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Period 5</t>
         </is>
       </c>
     </row>
@@ -551,26 +712,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>subject</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>minutes</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>date</t>
         </is>
@@ -590,7 +751,7 @@
       <c r="C2" t="n">
         <v>15</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D2" s="6" t="n">
         <v>46061</v>
       </c>
     </row>
@@ -608,7 +769,7 @@
       <c r="C3" t="n">
         <v>30</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D3" s="6" t="n">
         <v>46061</v>
       </c>
     </row>
@@ -626,7 +787,7 @@
       <c r="C4" t="n">
         <v>50</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="D4" s="6" t="n">
         <v>46068</v>
       </c>
     </row>
@@ -644,7 +805,7 @@
       <c r="C5" t="n">
         <v>16</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D5" s="6" t="n">
         <v>46069</v>
       </c>
     </row>
@@ -662,7 +823,7 @@
       <c r="C6" t="n">
         <v>21</v>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="D6" s="6" t="n">
         <v>46069</v>
       </c>
     </row>
@@ -680,8 +841,188 @@
       <c r="C7" t="n">
         <v>11</v>
       </c>
-      <c r="D7" s="3" t="n">
+      <c r="D7" s="6" t="n">
         <v>46082</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>mini pro</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>26</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>46083</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>php</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>26</v>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>46083</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>dcn</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>31</v>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>46083</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>dcn</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>31</v>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>46087</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>php</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>16</v>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>46087</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>mini pro</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>31</v>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>46087</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>mini pro</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>26</v>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>46089</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>dcn</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>51</v>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>46089</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>php</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>16</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>46089</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>php practical</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>21</v>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>46089</v>
       </c>
     </row>
   </sheetData>
@@ -695,21 +1036,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:C27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>habit</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>date</t>
         </is>
@@ -882,6 +1223,278 @@
       <c r="C11" t="inlineStr">
         <is>
           <t>2026-02-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>gym</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>water</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>food</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>sleep</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>gym</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>water</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>food</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>sleep</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-03-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>gym</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>water</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>food</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>sleep</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2026-03-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>gym</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>water</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>food</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>sleep</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2026-03-08</t>
         </is>
       </c>
     </row>
@@ -897,10 +1510,10 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:A5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>habit</t>
         </is>
@@ -945,16 +1558,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>subject</t>
         </is>
@@ -993,6 +1606,18 @@
       <c r="B4" t="inlineStr">
         <is>
           <t>dcn</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>php practical</t>
         </is>
       </c>
     </row>
@@ -1011,27 +1636,27 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>attendance</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>monthlygoal</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>minattendance</t>
         </is>
@@ -1069,36 +1694,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Created_Date</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Last_Reminded</t>
         </is>
@@ -1107,17 +1732,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>manishmanoj006@gmail.com</t>
+          <t>test@gmail.com</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>test@</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -1127,12 +1752,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-06</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-03-01 16:30:51</t>
+          <t>2026-03-08 13:51:57</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1769,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>aa</t>
+          <t>sun</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1154,17 +1779,17 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>2026-03-01 19:37:25</t>
+          <t>2026-03-08 16:40:33</t>
         </is>
       </c>
     </row>
@@ -1176,59 +1801,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ad</t>
+          <t>sum1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-08</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-03-01 12:48:55</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>manishmanoj006@gmail.com</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>re9</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Pending</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>2026-03-01 21:02:23</t>
+          <t>2026-03-08 16:41:39</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update attendance and habit fixes
</commit_message>
<xml_diff>
--- a/data/database.xlsx
+++ b/data/database.xlsx
@@ -22,9 +22,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -64,12 +63,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -461,7 +461,7 @@
           <t>manishmanoj006@gmail.com</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B2" s="3" t="n">
         <v>46086</v>
       </c>
       <c r="C2" t="inlineStr">
@@ -476,7 +476,7 @@
           <t>manishmanoj006@gmail.com</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B3" s="3" t="n">
         <v>46086</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -491,7 +491,7 @@
           <t>manishmanoj006@gmail.com</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B4" s="3" t="n">
         <v>46086</v>
       </c>
       <c r="C4" t="inlineStr">
@@ -506,7 +506,7 @@
           <t>manishmanoj006@gmail.com</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B5" s="3" t="n">
         <v>46086</v>
       </c>
       <c r="C5" t="inlineStr">
@@ -521,7 +521,7 @@
           <t>manishmanoj006@gmail.com</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B6" s="3" t="n">
         <v>46086</v>
       </c>
       <c r="C6" t="inlineStr">
@@ -536,7 +536,7 @@
           <t>manishmanoj006@gmail.com</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B7" s="3" t="n">
         <v>46087</v>
       </c>
       <c r="C7" t="inlineStr">
@@ -551,7 +551,7 @@
           <t>manishmanoj006@gmail.com</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B8" s="3" t="n">
         <v>46087</v>
       </c>
       <c r="C8" t="inlineStr">
@@ -566,7 +566,7 @@
           <t>manishmanoj006@gmail.com</t>
         </is>
       </c>
-      <c r="B9" s="2" t="n">
+      <c r="B9" s="3" t="n">
         <v>46087</v>
       </c>
       <c r="C9" t="inlineStr">
@@ -581,7 +581,7 @@
           <t>manishmanoj006@gmail.com</t>
         </is>
       </c>
-      <c r="B10" s="2" t="n">
+      <c r="B10" s="3" t="n">
         <v>46087</v>
       </c>
       <c r="C10" t="inlineStr">
@@ -596,7 +596,7 @@
           <t>manishmanoj006@gmail.com</t>
         </is>
       </c>
-      <c r="B11" s="2" t="n">
+      <c r="B11" s="3" t="n">
         <v>46087</v>
       </c>
       <c r="C11" t="inlineStr">
@@ -611,7 +611,7 @@
           <t>manishmanoj006@gmail.com</t>
         </is>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B12" s="3" t="n">
         <v>46088</v>
       </c>
       <c r="C12" t="inlineStr">
@@ -626,7 +626,7 @@
           <t>manishmanoj006@gmail.com</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n">
+      <c r="B13" s="3" t="n">
         <v>46088</v>
       </c>
       <c r="C13" t="inlineStr">
@@ -641,7 +641,7 @@
           <t>manishmanoj006@gmail.com</t>
         </is>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="B14" s="3" t="n">
         <v>46088</v>
       </c>
       <c r="C14" t="inlineStr">
@@ -656,7 +656,7 @@
           <t>manishmanoj006@gmail.com</t>
         </is>
       </c>
-      <c r="B15" s="2" t="n">
+      <c r="B15" s="3" t="n">
         <v>46089</v>
       </c>
       <c r="C15" t="inlineStr">
@@ -671,7 +671,7 @@
           <t>manishmanoj006@gmail.com</t>
         </is>
       </c>
-      <c r="B16" s="2" t="n">
+      <c r="B16" s="3" t="n">
         <v>46089</v>
       </c>
       <c r="C16" t="inlineStr">
@@ -686,7 +686,7 @@
           <t>manishmanoj006@gmail.com</t>
         </is>
       </c>
-      <c r="B17" s="2" t="n">
+      <c r="B17" s="3" t="n">
         <v>46089</v>
       </c>
       <c r="C17" t="inlineStr">
@@ -701,7 +701,7 @@
           <t>manishmanoj006@gmail.com</t>
         </is>
       </c>
-      <c r="B18" s="2" t="n">
+      <c r="B18" s="3" t="n">
         <v>46089</v>
       </c>
       <c r="C18" t="inlineStr">
@@ -716,7 +716,7 @@
           <t>manishmanoj006@gmail.com</t>
         </is>
       </c>
-      <c r="B19" s="2" t="n">
+      <c r="B19" s="3" t="n">
         <v>46089</v>
       </c>
       <c r="C19" t="inlineStr">
@@ -731,7 +731,7 @@
           <t>manishmanoj006@gmail.com</t>
         </is>
       </c>
-      <c r="B20" s="2" t="n">
+      <c r="B20" s="3" t="n">
         <v>46090</v>
       </c>
       <c r="C20" t="inlineStr">
@@ -746,7 +746,7 @@
           <t>testmail6869@gmail.com</t>
         </is>
       </c>
-      <c r="B21" s="2" t="n">
+      <c r="B21" s="3" t="n">
         <v>46090</v>
       </c>
       <c r="C21" t="inlineStr">
@@ -761,10 +761,25 @@
           <t>testmail6869@gmail.com</t>
         </is>
       </c>
-      <c r="B22" s="2" t="n">
+      <c r="B22" s="3" t="n">
         <v>46090</v>
       </c>
       <c r="C22" t="inlineStr">
+        <is>
+          <t>Period 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>manishmanoj006@gmail.com</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>46090</v>
+      </c>
+      <c r="C23" t="inlineStr">
         <is>
           <t>Period 2</t>
         </is>
@@ -1867,25 +1882,19 @@
           <t>manishmanoj006@gmail.com</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B2" t="n">
+        <v>2</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>manish</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>45</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>75</t>
-        </is>
+      <c r="D2" t="n">
+        <v>45</v>
+      </c>
+      <c r="E2" t="n">
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>